<commit_message>
Prepare publication workflow and Supplementary File S6
Add documented scripts, supplementary analyses, archived results and S6 resources. Apply MIT and CC BY 4.0 notices and preserve recorded file hashes.
</commit_message>
<xml_diff>
--- a/results/04_origin_assignment/step4_assignment_multilevel_macroregion_first.xlsx
+++ b/results/04_origin_assignment/step4_assignment_multilevel_macroregion_first.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="200">
   <si>
     <t xml:space="preserve">sample_id</t>
   </si>
@@ -472,15 +472,6 @@
     <t xml:space="preserve">Need &gt;= 300; have 200</t>
   </si>
   <si>
-    <t xml:space="preserve">Need &gt;= 300; have 198</t>
-  </si>
-  <si>
-    <t xml:space="preserve">low_gap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">posterior_gap&lt;0.25</t>
-  </si>
-  <si>
     <t xml:space="preserve">Moderate</t>
   </si>
   <si>
@@ -496,19 +487,19 @@
     <t xml:space="preserve">qc_dir</t>
   </si>
   <si>
-    <t xml:space="preserve">C:/Users/virgilio/Documents/GitHub/PESTFLY/PESTFLY_origin_tracing_MolEcolRes_publication_pipeline/results/01_qc</t>
+    <t xml:space="preserve">C:/Users/virgilio/Documents/GitHub/PESTFLY/000_REVISION_JPS_PESTFLY_origin_tracing_pipeline/results/01_qc</t>
   </si>
   <si>
     <t xml:space="preserve">step3_dir</t>
   </si>
   <si>
-    <t xml:space="preserve">C:/Users/virgilio/Documents/GitHub/PESTFLY/PESTFLY_origin_tracing_MolEcolRes_publication_pipeline/results/02_snp_panels</t>
+    <t xml:space="preserve">C:/Users/virgilio/Documents/GitHub/PESTFLY/000_REVISION_JPS_PESTFLY_origin_tracing_pipeline/results/02_snp_panels</t>
   </si>
   <si>
     <t xml:space="preserve">out_dir</t>
   </si>
   <si>
-    <t xml:space="preserve">C:/Users/virgilio/Documents/GitHub/PESTFLY/PESTFLY_origin_tracing_MolEcolRes_publication_pipeline/results/04_origin_assignment</t>
+    <t xml:space="preserve">C:/Users/virgilio/Documents/GitHub/PESTFLY/000_REVISION_JPS_PESTFLY_origin_tracing_pipeline/results/04_origin_assignment</t>
   </si>
   <si>
     <t xml:space="preserve">out_xlsx</t>
@@ -1322,7 +1313,7 @@
         <v>3</v>
       </c>
       <c r="O2" t="n">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="P2"/>
       <c r="Q2" t="s">
@@ -1484,7 +1475,7 @@
         <v>5</v>
       </c>
       <c r="O4" t="n">
-        <v>2883</v>
+        <v>2879</v>
       </c>
       <c r="P4"/>
       <c r="Q4" t="s">
@@ -1610,7 +1601,7 @@
         <v>6</v>
       </c>
       <c r="AD5" t="n">
-        <v>11069</v>
+        <v>11070</v>
       </c>
       <c r="AE5" t="s">
         <v>40</v>
@@ -1717,7 +1708,7 @@
         <v>6</v>
       </c>
       <c r="AD6" t="n">
-        <v>11071</v>
+        <v>11070</v>
       </c>
       <c r="AE6" t="s">
         <v>40</v>
@@ -1824,7 +1815,7 @@
         <v>6</v>
       </c>
       <c r="AD7" t="n">
-        <v>11074</v>
+        <v>11075</v>
       </c>
       <c r="AE7" t="s">
         <v>40</v>
@@ -2038,7 +2029,7 @@
         <v>6</v>
       </c>
       <c r="AD9" t="n">
-        <v>11060</v>
+        <v>11059</v>
       </c>
       <c r="AE9" t="s">
         <v>40</v>
@@ -2100,7 +2091,7 @@
         <v>6</v>
       </c>
       <c r="O10" t="n">
-        <v>11064</v>
+        <v>11063</v>
       </c>
       <c r="P10" t="s">
         <v>56</v>
@@ -2118,22 +2109,22 @@
         <v>11001</v>
       </c>
       <c r="U10" t="n">
-        <v>0.999999999980881</v>
+        <v>0.999996129644487</v>
       </c>
       <c r="V10" t="n">
-        <v>0.999999999961762</v>
+        <v>0.999992259288973</v>
       </c>
       <c r="W10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X10" t="n">
         <v>0.666666666666667</v>
-      </c>
-      <c r="X10" t="n">
-        <v>1</v>
       </c>
       <c r="Y10" t="n">
         <v>0.5</v>
       </c>
       <c r="Z10" t="n">
-        <v>5000</v>
+        <v>11001</v>
       </c>
       <c r="AA10" t="n">
         <v>6</v>
@@ -2252,7 +2243,7 @@
         <v>6</v>
       </c>
       <c r="AD11" t="n">
-        <v>11073</v>
+        <v>11074</v>
       </c>
       <c r="AE11" t="s">
         <v>40</v>
@@ -2359,7 +2350,7 @@
         <v>6</v>
       </c>
       <c r="AD12" t="n">
-        <v>11076</v>
+        <v>11077</v>
       </c>
       <c r="AE12" t="s">
         <v>40</v>
@@ -2439,10 +2430,10 @@
         <v>11001</v>
       </c>
       <c r="U13" t="n">
-        <v>0.984124827168232</v>
+        <v>0.931552139662621</v>
       </c>
       <c r="V13" t="n">
-        <v>0.968249654336464</v>
+        <v>0.863104279325242</v>
       </c>
       <c r="W13" t="n">
         <v>0.333333333333333</v>
@@ -2466,7 +2457,7 @@
         <v>6</v>
       </c>
       <c r="AD13" t="n">
-        <v>10993</v>
+        <v>10992</v>
       </c>
       <c r="AE13" t="s">
         <v>40</v>
@@ -2680,7 +2671,7 @@
         <v>6</v>
       </c>
       <c r="AD15" t="n">
-        <v>10982</v>
+        <v>10981</v>
       </c>
       <c r="AE15" t="s">
         <v>40</v>
@@ -2742,7 +2733,7 @@
         <v>6</v>
       </c>
       <c r="O16" t="n">
-        <v>11063</v>
+        <v>11062</v>
       </c>
       <c r="P16" t="s">
         <v>63</v>
@@ -2787,7 +2778,7 @@
         <v>6</v>
       </c>
       <c r="AD16" t="n">
-        <v>10974</v>
+        <v>10975</v>
       </c>
       <c r="AE16" t="s">
         <v>40</v>
@@ -2894,7 +2885,7 @@
         <v>6</v>
       </c>
       <c r="AD17" t="n">
-        <v>11073</v>
+        <v>11072</v>
       </c>
       <c r="AE17" t="s">
         <v>40</v>
@@ -2974,13 +2965,13 @@
         <v>11001</v>
       </c>
       <c r="U18" t="n">
-        <v>0.999999962646162</v>
+        <v>0.999999872479476</v>
       </c>
       <c r="V18" t="n">
-        <v>0.999999925292324</v>
+        <v>0.999999744958951</v>
       </c>
       <c r="W18" t="n">
-        <v>0.5</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="X18" t="n">
         <v>1</v>
@@ -2989,7 +2980,7 @@
         <v>0.5</v>
       </c>
       <c r="Z18" t="n">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="AA18" t="n">
         <v>6</v>
@@ -3170,7 +3161,7 @@
         <v>7</v>
       </c>
       <c r="O20" t="n">
-        <v>11070</v>
+        <v>11071</v>
       </c>
       <c r="P20" t="s">
         <v>63</v>
@@ -3322,7 +3313,7 @@
         <v>6</v>
       </c>
       <c r="AD21" t="n">
-        <v>10984</v>
+        <v>10983</v>
       </c>
       <c r="AE21" t="s">
         <v>40</v>
@@ -13935,13 +13926,13 @@
         <v>44</v>
       </c>
       <c r="H292" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000179851080284381</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000107548334203744</v>
       </c>
       <c r="I292" t="n">
         <v>1</v>
       </c>
       <c r="J292" t="n">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="K292" t="s">
         <v>47</v>
@@ -13982,7 +13973,7 @@
         <v>1</v>
       </c>
       <c r="J293" t="n">
-        <v>1578</v>
+        <v>1580</v>
       </c>
       <c r="K293" t="s">
         <v>47</v>
@@ -14023,7 +14014,7 @@
         <v>1</v>
       </c>
       <c r="J294" t="n">
-        <v>1415</v>
+        <v>1416</v>
       </c>
       <c r="K294" t="s">
         <v>47</v>
@@ -14146,7 +14137,7 @@
         <v>1</v>
       </c>
       <c r="J297" t="n">
-        <v>4994</v>
+        <v>4993</v>
       </c>
       <c r="K297" t="s">
         <v>47</v>
@@ -14837,13 +14828,13 @@
         <v>44</v>
       </c>
       <c r="H314" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000111349874739484</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000404353949313298</v>
       </c>
       <c r="I314" t="n">
         <v>1</v>
       </c>
       <c r="J314" t="n">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="K314" t="s">
         <v>47</v>
@@ -14884,7 +14875,7 @@
         <v>1</v>
       </c>
       <c r="J315" t="n">
-        <v>2936</v>
+        <v>2934</v>
       </c>
       <c r="K315" t="s">
         <v>47</v>
@@ -14925,7 +14916,7 @@
         <v>1</v>
       </c>
       <c r="J316" t="n">
-        <v>2585</v>
+        <v>2581</v>
       </c>
       <c r="K316" t="s">
         <v>47</v>
@@ -15253,7 +15244,7 @@
         <v>1</v>
       </c>
       <c r="J324" t="n">
-        <v>9985</v>
+        <v>9986</v>
       </c>
       <c r="K324" t="s">
         <v>47</v>
@@ -15739,13 +15730,13 @@
         <v>44</v>
       </c>
       <c r="H336" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000117148920508671</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000447443108134209</v>
       </c>
       <c r="I336" t="n">
         <v>1</v>
       </c>
       <c r="J336" t="n">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="K336" t="s">
         <v>47</v>
@@ -15827,7 +15818,7 @@
         <v>1</v>
       </c>
       <c r="J338" t="n">
-        <v>2883</v>
+        <v>2879</v>
       </c>
       <c r="K338" t="s">
         <v>47</v>
@@ -15909,7 +15900,7 @@
         <v>1</v>
       </c>
       <c r="J340" t="n">
-        <v>11064</v>
+        <v>11063</v>
       </c>
       <c r="K340" t="s">
         <v>47</v>
@@ -16155,7 +16146,7 @@
         <v>1</v>
       </c>
       <c r="J346" t="n">
-        <v>11070</v>
+        <v>11071</v>
       </c>
       <c r="K346" t="s">
         <v>47</v>
@@ -16401,7 +16392,7 @@
         <v>1</v>
       </c>
       <c r="J352" t="n">
-        <v>11063</v>
+        <v>11062</v>
       </c>
       <c r="K352" t="s">
         <v>47</v>
@@ -16786,7 +16777,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000117148920508671</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000447443108134209</v>
       </c>
       <c r="N6" t="n">
         <v>1</v>
@@ -16798,7 +16789,7 @@
         <v>48</v>
       </c>
       <c r="Q6" t="n">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="R6" t="s">
         <v>48</v>
@@ -16910,7 +16901,7 @@
         <v>48</v>
       </c>
       <c r="Q8" t="n">
-        <v>2883</v>
+        <v>2879</v>
       </c>
       <c r="R8" t="s">
         <v>48</v>
@@ -17022,7 +17013,7 @@
         <v>48</v>
       </c>
       <c r="Q10" t="n">
-        <v>11064</v>
+        <v>11063</v>
       </c>
       <c r="R10" t="s">
         <v>48</v>
@@ -17358,7 +17349,7 @@
         <v>48</v>
       </c>
       <c r="Q16" t="n">
-        <v>11070</v>
+        <v>11071</v>
       </c>
       <c r="R16" t="s">
         <v>48</v>
@@ -17694,7 +17685,7 @@
         <v>48</v>
       </c>
       <c r="Q22" t="n">
-        <v>11063</v>
+        <v>11062</v>
       </c>
       <c r="R22" t="s">
         <v>48</v>
@@ -21302,7 +21293,7 @@
       <c r="H114"/>
       <c r="I114"/>
       <c r="J114" t="n">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K114" t="s">
         <v>90</v>
@@ -21311,7 +21302,7 @@
         <v>91</v>
       </c>
       <c r="M114" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="115">
@@ -21519,7 +21510,7 @@
       <c r="H121"/>
       <c r="I121"/>
       <c r="J121" t="n">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K121" t="s">
         <v>90</v>
@@ -21528,7 +21519,7 @@
         <v>91</v>
       </c>
       <c r="M121" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="122">
@@ -21548,16 +21539,16 @@
         <v>63</v>
       </c>
       <c r="F122" t="n">
-        <v>0.999884456822819</v>
+        <v>0.99999985164328</v>
       </c>
       <c r="G122" t="s">
         <v>56</v>
       </c>
       <c r="H122" t="n">
-        <v>0.000115543177180849</v>
+        <v>0.000000148356719675843</v>
       </c>
       <c r="I122" t="n">
-        <v>0.999768913645638</v>
+        <v>0.999999703286561</v>
       </c>
       <c r="J122" t="n">
         <v>499</v>
@@ -21589,28 +21580,28 @@
         <v>56</v>
       </c>
       <c r="F123" t="n">
-        <v>0.514399086971685</v>
+        <v>0.986368354895643</v>
       </c>
       <c r="G123" t="s">
         <v>63</v>
       </c>
       <c r="H123" t="n">
-        <v>0.485600913028314</v>
+        <v>0.0136316451043572</v>
       </c>
       <c r="I123" t="n">
-        <v>0.028798173943371</v>
+        <v>0.972736709791286</v>
       </c>
       <c r="J123" t="n">
         <v>500</v>
       </c>
       <c r="K123" t="s">
-        <v>90</v>
+        <v>47</v>
       </c>
       <c r="L123" t="s">
-        <v>151</v>
+        <v>48</v>
       </c>
       <c r="M123" t="s">
-        <v>152</v>
+        <v>112</v>
       </c>
     </row>
     <row r="124">
@@ -21630,16 +21621,16 @@
         <v>56</v>
       </c>
       <c r="F124" t="n">
-        <v>0.999999995918527</v>
+        <v>0.999999998993172</v>
       </c>
       <c r="G124" t="s">
         <v>63</v>
       </c>
       <c r="H124" t="n">
-        <v>0.00000000408147266530867</v>
+        <v>0.00000000100682814337977</v>
       </c>
       <c r="I124" t="n">
-        <v>0.999999991837055</v>
+        <v>0.999999997986344</v>
       </c>
       <c r="J124" t="n">
         <v>500</v>
@@ -21671,16 +21662,16 @@
         <v>56</v>
       </c>
       <c r="F125" t="n">
-        <v>0.999999984302851</v>
+        <v>0.999999999354608</v>
       </c>
       <c r="G125" t="s">
         <v>63</v>
       </c>
       <c r="H125" t="n">
-        <v>0.0000000156971494403564</v>
+        <v>0.000000000645391709809303</v>
       </c>
       <c r="I125" t="n">
-        <v>0.999999968605701</v>
+        <v>0.999999998709217</v>
       </c>
       <c r="J125" t="n">
         <v>498</v>
@@ -21712,16 +21703,16 @@
         <v>63</v>
       </c>
       <c r="F126" t="n">
-        <v>0.999997478629904</v>
+        <v>0.99998793723351</v>
       </c>
       <c r="G126" t="s">
         <v>56</v>
       </c>
       <c r="H126" t="n">
-        <v>0.00000252137009613668</v>
+        <v>0.0000120627664897486</v>
       </c>
       <c r="I126" t="n">
-        <v>0.999994957259808</v>
+        <v>0.999975874467021</v>
       </c>
       <c r="J126" t="n">
         <v>498</v>
@@ -21753,16 +21744,16 @@
         <v>63</v>
       </c>
       <c r="F127" t="n">
-        <v>0.999888135315278</v>
+        <v>0.999992470084371</v>
       </c>
       <c r="G127" t="s">
         <v>56</v>
       </c>
       <c r="H127" t="n">
-        <v>0.000111864684722229</v>
+        <v>0.00000752991562868548</v>
       </c>
       <c r="I127" t="n">
-        <v>0.999776270630556</v>
+        <v>0.999984940168743</v>
       </c>
       <c r="J127" t="n">
         <v>500</v>
@@ -21794,16 +21785,16 @@
         <v>56</v>
       </c>
       <c r="F128" t="n">
-        <v>0.999999971342217</v>
+        <v>0.999999748743565</v>
       </c>
       <c r="G128" t="s">
         <v>63</v>
       </c>
       <c r="H128" t="n">
-        <v>0.0000000286577829373809</v>
+        <v>0.000000251256434890343</v>
       </c>
       <c r="I128" t="n">
-        <v>0.999999942684434</v>
+        <v>0.99999949748713</v>
       </c>
       <c r="J128" t="n">
         <v>500</v>
@@ -21835,16 +21826,16 @@
         <v>63</v>
       </c>
       <c r="F129" t="n">
-        <v>0.999999988758994</v>
+        <v>0.999999999746791</v>
       </c>
       <c r="G129" t="s">
         <v>56</v>
       </c>
       <c r="H129" t="n">
-        <v>0.0000000112410065308877</v>
+        <v>0.000000000253208589460165</v>
       </c>
       <c r="I129" t="n">
-        <v>0.999999977517987</v>
+        <v>0.999999999493583</v>
       </c>
       <c r="J129" t="n">
         <v>500</v>
@@ -21876,16 +21867,16 @@
         <v>56</v>
       </c>
       <c r="F130" t="n">
-        <v>0.999999999999972</v>
+        <v>0.999999999999998</v>
       </c>
       <c r="G130" t="s">
         <v>63</v>
       </c>
       <c r="H130" t="n">
-        <v>0.0000000000000284210719943733</v>
+        <v>0.00000000000000165026417998991</v>
       </c>
       <c r="I130" t="n">
-        <v>0.999999999999943</v>
+        <v>0.999999999999997</v>
       </c>
       <c r="J130" t="n">
         <v>499</v>
@@ -21917,16 +21908,16 @@
         <v>56</v>
       </c>
       <c r="F131" t="n">
-        <v>0.999999645606447</v>
+        <v>0.999983291284812</v>
       </c>
       <c r="G131" t="s">
         <v>63</v>
       </c>
       <c r="H131" t="n">
-        <v>0.000000354393552882007</v>
+        <v>0.0000167087151876206</v>
       </c>
       <c r="I131" t="n">
-        <v>0.999999291212894</v>
+        <v>0.999966582569625</v>
       </c>
       <c r="J131" t="n">
         <v>500</v>
@@ -21958,16 +21949,16 @@
         <v>56</v>
       </c>
       <c r="F132" t="n">
-        <v>0.5782376755927</v>
+        <v>0.825736625370286</v>
       </c>
       <c r="G132" t="s">
         <v>63</v>
       </c>
       <c r="H132" t="n">
-        <v>0.4217623244073</v>
+        <v>0.174263374629714</v>
       </c>
       <c r="I132" t="n">
-        <v>0.156475351185401</v>
+        <v>0.651473250740572</v>
       </c>
       <c r="J132" t="n">
         <v>499</v>
@@ -21976,10 +21967,10 @@
         <v>90</v>
       </c>
       <c r="L132" t="s">
-        <v>151</v>
+        <v>48</v>
       </c>
       <c r="M132" t="s">
-        <v>152</v>
+        <v>112</v>
       </c>
     </row>
     <row r="133">
@@ -21999,16 +21990,16 @@
         <v>63</v>
       </c>
       <c r="F133" t="n">
-        <v>0.999999867838824</v>
+        <v>0.999999512681129</v>
       </c>
       <c r="G133" t="s">
         <v>56</v>
       </c>
       <c r="H133" t="n">
-        <v>0.000000132161176349673</v>
+        <v>0.000000487318870690241</v>
       </c>
       <c r="I133" t="n">
-        <v>0.999999735677647</v>
+        <v>0.999999025362259</v>
       </c>
       <c r="J133" t="n">
         <v>498</v>
@@ -22040,16 +22031,16 @@
         <v>63</v>
       </c>
       <c r="F134" t="n">
-        <v>0.999940344125702</v>
+        <v>0.999956693865265</v>
       </c>
       <c r="G134" t="s">
         <v>56</v>
       </c>
       <c r="H134" t="n">
-        <v>0.0000596558742976888</v>
+        <v>0.0000433061347345979</v>
       </c>
       <c r="I134" t="n">
-        <v>0.999880688251405</v>
+        <v>0.999913387730531</v>
       </c>
       <c r="J134" t="n">
         <v>997</v>
@@ -22081,16 +22072,16 @@
         <v>63</v>
       </c>
       <c r="F135" t="n">
-        <v>0.999989854595779</v>
+        <v>0.999998615945972</v>
       </c>
       <c r="G135" t="s">
         <v>56</v>
       </c>
       <c r="H135" t="n">
-        <v>0.0000101454042205134</v>
+        <v>0.00000138405402826924</v>
       </c>
       <c r="I135" t="n">
-        <v>0.999979709191559</v>
+        <v>0.999997231891943</v>
       </c>
       <c r="J135" t="n">
         <v>1000</v>
@@ -22122,16 +22113,16 @@
         <v>56</v>
       </c>
       <c r="F136" t="n">
-        <v>0.999999999999997</v>
+        <v>1</v>
       </c>
       <c r="G136" t="s">
         <v>63</v>
       </c>
       <c r="H136" t="n">
-        <v>0.00000000000000282414484803873</v>
+        <v>0.000000000000000319149483362032</v>
       </c>
       <c r="I136" t="n">
-        <v>0.999999999999994</v>
+        <v>0.999999999999999</v>
       </c>
       <c r="J136" t="n">
         <v>999</v>
@@ -22163,16 +22154,16 @@
         <v>56</v>
       </c>
       <c r="F137" t="n">
-        <v>0.999999981421179</v>
+        <v>0.999999987202574</v>
       </c>
       <c r="G137" t="s">
         <v>63</v>
       </c>
       <c r="H137" t="n">
-        <v>0.0000000185788215532055</v>
+        <v>0.0000000127974259653129</v>
       </c>
       <c r="I137" t="n">
-        <v>0.999999962842357</v>
+        <v>0.999999974405148</v>
       </c>
       <c r="J137" t="n">
         <v>997</v>
@@ -22204,16 +22195,16 @@
         <v>63</v>
       </c>
       <c r="F138" t="n">
-        <v>0.999999999741183</v>
+        <v>0.999999999984949</v>
       </c>
       <c r="G138" t="s">
         <v>56</v>
       </c>
       <c r="H138" t="n">
-        <v>0.000000000258817067141481</v>
+        <v>0.0000000000150511370107944</v>
       </c>
       <c r="I138" t="n">
-        <v>0.999999999482366</v>
+        <v>0.999999999969898</v>
       </c>
       <c r="J138" t="n">
         <v>998</v>
@@ -22251,7 +22242,7 @@
         <v>56</v>
       </c>
       <c r="H139" t="n">
-        <v>0.0000000000000000768657722366552</v>
+        <v>0.000000000000000147207162912354</v>
       </c>
       <c r="I139" t="n">
         <v>1</v>
@@ -22286,16 +22277,16 @@
         <v>56</v>
       </c>
       <c r="F140" t="n">
-        <v>1</v>
+        <v>0.999999999999989</v>
       </c>
       <c r="G140" t="s">
         <v>63</v>
       </c>
       <c r="H140" t="n">
-        <v>0.000000000000000230067671333</v>
+        <v>0.0000000000000110268438194531</v>
       </c>
       <c r="I140" t="n">
-        <v>1</v>
+        <v>0.999999999999978</v>
       </c>
       <c r="J140" t="n">
         <v>999</v>
@@ -22333,7 +22324,7 @@
         <v>56</v>
       </c>
       <c r="H141" t="n">
-        <v>0.00000000000000000119601640634199</v>
+        <v>0.000000000000000000165495897256451</v>
       </c>
       <c r="I141" t="n">
         <v>1</v>
@@ -22374,7 +22365,7 @@
         <v>63</v>
       </c>
       <c r="H142" t="n">
-        <v>0.00000000000000000000000000000244663612775688</v>
+        <v>0.00000000000000000000000000000599638609525546</v>
       </c>
       <c r="I142" t="n">
         <v>1</v>
@@ -22409,16 +22400,16 @@
         <v>56</v>
       </c>
       <c r="F143" t="n">
-        <v>0.999997989735381</v>
+        <v>0.999832179496809</v>
       </c>
       <c r="G143" t="s">
         <v>63</v>
       </c>
       <c r="H143" t="n">
-        <v>0.00000201026461955972</v>
+        <v>0.000167820503191378</v>
       </c>
       <c r="I143" t="n">
-        <v>0.999995979470761</v>
+        <v>0.999664358993617</v>
       </c>
       <c r="J143" t="n">
         <v>1000</v>
@@ -22450,16 +22441,16 @@
         <v>63</v>
       </c>
       <c r="F144" t="n">
-        <v>0.999999988515342</v>
+        <v>0.999999999393501</v>
       </c>
       <c r="G144" t="s">
         <v>56</v>
       </c>
       <c r="H144" t="n">
-        <v>0.0000000114846575180551</v>
+        <v>0.000000000606499040725213</v>
       </c>
       <c r="I144" t="n">
-        <v>0.999999977030685</v>
+        <v>0.999999998787002</v>
       </c>
       <c r="J144" t="n">
         <v>998</v>
@@ -22491,16 +22482,16 @@
         <v>63</v>
       </c>
       <c r="F145" t="n">
-        <v>0.999999999999784</v>
+        <v>0.999999999999083</v>
       </c>
       <c r="G145" t="s">
         <v>56</v>
       </c>
       <c r="H145" t="n">
-        <v>0.000000000000215628985289583</v>
+        <v>0.000000000000917597173547056</v>
       </c>
       <c r="I145" t="n">
-        <v>0.999999999999569</v>
+        <v>0.999999999998165</v>
       </c>
       <c r="J145" t="n">
         <v>997</v>
@@ -22532,16 +22523,16 @@
         <v>63</v>
       </c>
       <c r="F146" t="n">
-        <v>0.999991157821192</v>
+        <v>0.999999737388515</v>
       </c>
       <c r="G146" t="s">
         <v>56</v>
       </c>
       <c r="H146" t="n">
-        <v>0.00000884217880780963</v>
+        <v>0.000000262611485251789</v>
       </c>
       <c r="I146" t="n">
-        <v>0.999982315642384</v>
+        <v>0.999999474777029</v>
       </c>
       <c r="J146" t="n">
         <v>1996</v>
@@ -22573,16 +22564,16 @@
         <v>63</v>
       </c>
       <c r="F147" t="n">
-        <v>0.999999999996219</v>
+        <v>0.999999999999992</v>
       </c>
       <c r="G147" t="s">
         <v>56</v>
       </c>
       <c r="H147" t="n">
-        <v>0.00000000000378091049331874</v>
+        <v>0.00000000000000795028781124339</v>
       </c>
       <c r="I147" t="n">
-        <v>0.999999999992438</v>
+        <v>0.999999999999984</v>
       </c>
       <c r="J147" t="n">
         <v>1998</v>
@@ -22614,16 +22605,16 @@
         <v>56</v>
       </c>
       <c r="F148" t="n">
-        <v>0.999999999999647</v>
+        <v>0.999999999338462</v>
       </c>
       <c r="G148" t="s">
         <v>63</v>
       </c>
       <c r="H148" t="n">
-        <v>0.000000000000352753890491246</v>
+        <v>0.000000000661538117772601</v>
       </c>
       <c r="I148" t="n">
-        <v>0.999999999999294</v>
+        <v>0.999999998676924</v>
       </c>
       <c r="J148" t="n">
         <v>1998</v>
@@ -22652,25 +22643,25 @@
         <v>68</v>
       </c>
       <c r="E149" t="s">
+        <v>63</v>
+      </c>
+      <c r="F149" t="n">
+        <v>0.996798125612403</v>
+      </c>
+      <c r="G149" t="s">
         <v>56</v>
       </c>
-      <c r="F149" t="n">
-        <v>0.853894462978456</v>
-      </c>
-      <c r="G149" t="s">
-        <v>63</v>
-      </c>
       <c r="H149" t="n">
-        <v>0.146105537021544</v>
+        <v>0.00320187438759712</v>
       </c>
       <c r="I149" t="n">
-        <v>0.707788925956912</v>
+        <v>0.993596251224806</v>
       </c>
       <c r="J149" t="n">
         <v>1996</v>
       </c>
       <c r="K149" t="s">
-        <v>153</v>
+        <v>47</v>
       </c>
       <c r="L149" t="s">
         <v>48</v>
@@ -22696,16 +22687,16 @@
         <v>63</v>
       </c>
       <c r="F150" t="n">
-        <v>0.999999999999961</v>
+        <v>1</v>
       </c>
       <c r="G150" t="s">
         <v>56</v>
       </c>
       <c r="H150" t="n">
-        <v>0.0000000000000390855679457426</v>
+        <v>0.0000000000000000163062811380108</v>
       </c>
       <c r="I150" t="n">
-        <v>0.999999999999922</v>
+        <v>1</v>
       </c>
       <c r="J150" t="n">
         <v>1998</v>
@@ -22743,7 +22734,7 @@
         <v>56</v>
       </c>
       <c r="H151" t="n">
-        <v>0.000000000000000000000000000000000274677176862838</v>
+        <v>0.00000000000000000000000000000000000925976910403446</v>
       </c>
       <c r="I151" t="n">
         <v>1</v>
@@ -22784,7 +22775,7 @@
         <v>63</v>
       </c>
       <c r="H152" t="n">
-        <v>0.00000000000000000000158440123330592</v>
+        <v>0.0000000000000000000000766120536722968</v>
       </c>
       <c r="I152" t="n">
         <v>1</v>
@@ -22825,7 +22816,7 @@
         <v>56</v>
       </c>
       <c r="H153" t="n">
-        <v>0.0000000000000000000000000000000000000000448252564397843</v>
+        <v>0.0000000000000000000000000000000000000000000174546640152097</v>
       </c>
       <c r="I153" t="n">
         <v>1</v>
@@ -22866,7 +22857,7 @@
         <v>63</v>
       </c>
       <c r="H154" t="n">
-        <v>0.00000000000000000000000000000000000000000000000143615820709829</v>
+        <v>0.0000000000000000000000000000000000000000000000064943934543359</v>
       </c>
       <c r="I154" t="n">
         <v>1</v>
@@ -22901,16 +22892,16 @@
         <v>56</v>
       </c>
       <c r="F155" t="n">
-        <v>0.99999999937521</v>
+        <v>0.999996050249059</v>
       </c>
       <c r="G155" t="s">
         <v>63</v>
       </c>
       <c r="H155" t="n">
-        <v>0.000000000624789833669235</v>
+        <v>0.0000039497509404763</v>
       </c>
       <c r="I155" t="n">
-        <v>0.99999999875042</v>
+        <v>0.999992100498119</v>
       </c>
       <c r="J155" t="n">
         <v>1999</v>
@@ -22948,13 +22939,13 @@
         <v>56</v>
       </c>
       <c r="H156" t="n">
-        <v>0.00000000000000039641310401561</v>
+        <v>0.000000000000000000798863572260363</v>
       </c>
       <c r="I156" t="n">
-        <v>0.999999999999999</v>
+        <v>1</v>
       </c>
       <c r="J156" t="n">
-        <v>1996</v>
+        <v>1995</v>
       </c>
       <c r="K156" t="s">
         <v>47</v>
@@ -22989,10 +22980,10 @@
         <v>56</v>
       </c>
       <c r="H157" t="n">
-        <v>0.000000000000000424062565052894</v>
+        <v>0.0000000000000000690819333667313</v>
       </c>
       <c r="I157" t="n">
-        <v>0.999999999999999</v>
+        <v>1</v>
       </c>
       <c r="J157" t="n">
         <v>1993</v>
@@ -23024,19 +23015,19 @@
         <v>56</v>
       </c>
       <c r="F158" t="n">
-        <v>0.999999138597232</v>
+        <v>0.99999994929767</v>
       </c>
       <c r="G158" t="s">
         <v>63</v>
       </c>
       <c r="H158" t="n">
-        <v>0.000000861402768244823</v>
+        <v>0.0000000507023299084888</v>
       </c>
       <c r="I158" t="n">
-        <v>0.999998277194463</v>
+        <v>0.99999989859534</v>
       </c>
       <c r="J158" t="n">
-        <v>4994</v>
+        <v>4996</v>
       </c>
       <c r="K158" t="s">
         <v>47</v>
@@ -23065,19 +23056,19 @@
         <v>56</v>
       </c>
       <c r="F159" t="n">
-        <v>0.999959369338436</v>
+        <v>0.999987037211283</v>
       </c>
       <c r="G159" t="s">
         <v>63</v>
       </c>
       <c r="H159" t="n">
-        <v>0.0000406306615639706</v>
+        <v>0.0000129627887169618</v>
       </c>
       <c r="I159" t="n">
-        <v>0.999918738676872</v>
+        <v>0.999974074422566</v>
       </c>
       <c r="J159" t="n">
-        <v>4997</v>
+        <v>4998</v>
       </c>
       <c r="K159" t="s">
         <v>47</v>
@@ -23112,10 +23103,10 @@
         <v>63</v>
       </c>
       <c r="H160" t="n">
-        <v>0.0000000000000000533131094578182</v>
+        <v>0.000000000000000353314182657466</v>
       </c>
       <c r="I160" t="n">
-        <v>1</v>
+        <v>0.999999999999999</v>
       </c>
       <c r="J160" t="n">
         <v>4996</v>
@@ -23147,19 +23138,19 @@
         <v>63</v>
       </c>
       <c r="F161" t="n">
-        <v>0.999905316169232</v>
+        <v>0.999994375381017</v>
       </c>
       <c r="G161" t="s">
         <v>56</v>
       </c>
       <c r="H161" t="n">
-        <v>0.0000946838307684642</v>
+        <v>0.00000562461898328003</v>
       </c>
       <c r="I161" t="n">
-        <v>0.999810632338463</v>
+        <v>0.999988750762034</v>
       </c>
       <c r="J161" t="n">
-        <v>4993</v>
+        <v>4995</v>
       </c>
       <c r="K161" t="s">
         <v>47</v>
@@ -23194,7 +23185,7 @@
         <v>56</v>
       </c>
       <c r="H162" t="n">
-        <v>0.00000000000000000000000000000000000000000271181383840276</v>
+        <v>0.0000000000000000000000000000000000000000000420774438740403</v>
       </c>
       <c r="I162" t="n">
         <v>1</v>
@@ -23235,7 +23226,7 @@
         <v>56</v>
       </c>
       <c r="H163" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000000435149975249912</v>
+        <v>0.000000000000000000000000000000000000000000000000000000000000018445628230255</v>
       </c>
       <c r="I163" t="n">
         <v>1</v>
@@ -23276,13 +23267,13 @@
         <v>63</v>
       </c>
       <c r="H164" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000351115905062262</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000928233978524381</v>
       </c>
       <c r="I164" t="n">
         <v>1</v>
       </c>
       <c r="J164" t="n">
-        <v>4995</v>
+        <v>4996</v>
       </c>
       <c r="K164" t="s">
         <v>47</v>
@@ -23317,13 +23308,13 @@
         <v>56</v>
       </c>
       <c r="H165" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000071439381147102</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000036009379481891</v>
       </c>
       <c r="I165" t="n">
         <v>1</v>
       </c>
       <c r="J165" t="n">
-        <v>4993</v>
+        <v>4994</v>
       </c>
       <c r="K165" t="s">
         <v>47</v>
@@ -23358,7 +23349,7 @@
         <v>63</v>
       </c>
       <c r="H166" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000985484802002937</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000745716249585789</v>
       </c>
       <c r="I166" t="n">
         <v>1</v>
@@ -23393,16 +23384,16 @@
         <v>56</v>
       </c>
       <c r="F167" t="n">
-        <v>0.96745022720156</v>
+        <v>0.99676331665444</v>
       </c>
       <c r="G167" t="s">
         <v>63</v>
       </c>
       <c r="H167" t="n">
-        <v>0.0325497727984397</v>
+        <v>0.00323668334556016</v>
       </c>
       <c r="I167" t="n">
-        <v>0.934900454403121</v>
+        <v>0.99352663330888</v>
       </c>
       <c r="J167" t="n">
         <v>4999</v>
@@ -23440,13 +23431,13 @@
         <v>56</v>
       </c>
       <c r="H168" t="n">
-        <v>0.00000000000000000000000000000000000000798594886323024</v>
+        <v>0.000000000000000000000000000000000000000410735079436623</v>
       </c>
       <c r="I168" t="n">
         <v>1</v>
       </c>
       <c r="J168" t="n">
-        <v>4992</v>
+        <v>4991</v>
       </c>
       <c r="K168" t="s">
         <v>47</v>
@@ -23481,7 +23472,7 @@
         <v>56</v>
       </c>
       <c r="H169" t="n">
-        <v>0.000000000000000000000000000000000000000000134004560072763</v>
+        <v>0.00000000000000000000000000000000000000000000127845488963131</v>
       </c>
       <c r="I169" t="n">
         <v>1</v>
@@ -23522,7 +23513,7 @@
         <v>63</v>
       </c>
       <c r="H170" t="n">
-        <v>0.00000000000000000000000184142693143148</v>
+        <v>0.0000000000000000000000523986647432691</v>
       </c>
       <c r="I170" t="n">
         <v>1</v>
@@ -23554,31 +23545,31 @@
         <v>59</v>
       </c>
       <c r="E171" t="s">
+        <v>63</v>
+      </c>
+      <c r="F171" t="n">
+        <v>0.999999494778271</v>
+      </c>
+      <c r="G171" t="s">
         <v>56</v>
       </c>
-      <c r="F171" t="n">
-        <v>0.590381200154785</v>
-      </c>
-      <c r="G171" t="s">
-        <v>63</v>
-      </c>
       <c r="H171" t="n">
-        <v>0.409618799845215</v>
+        <v>0.000000505221728975601</v>
       </c>
       <c r="I171" t="n">
-        <v>0.180762400309569</v>
+        <v>0.999998989556542</v>
       </c>
       <c r="J171" t="n">
         <v>9987</v>
       </c>
       <c r="K171" t="s">
-        <v>90</v>
+        <v>47</v>
       </c>
       <c r="L171" t="s">
-        <v>151</v>
+        <v>48</v>
       </c>
       <c r="M171" t="s">
-        <v>152</v>
+        <v>112</v>
       </c>
     </row>
     <row r="172">
@@ -23598,19 +23589,19 @@
         <v>63</v>
       </c>
       <c r="F172" t="n">
-        <v>0.999999999978454</v>
+        <v>0.999999997271629</v>
       </c>
       <c r="G172" t="s">
         <v>56</v>
       </c>
       <c r="H172" t="n">
-        <v>0.0000000000215462098745621</v>
+        <v>0.00000000272837073703177</v>
       </c>
       <c r="I172" t="n">
-        <v>0.999999999956907</v>
+        <v>0.999999994543259</v>
       </c>
       <c r="J172" t="n">
-        <v>9994</v>
+        <v>9993</v>
       </c>
       <c r="K172" t="s">
         <v>47</v>
@@ -23639,16 +23630,16 @@
         <v>63</v>
       </c>
       <c r="F173" t="n">
-        <v>0.999999999988995</v>
+        <v>0.999999999999993</v>
       </c>
       <c r="G173" t="s">
         <v>56</v>
       </c>
       <c r="H173" t="n">
-        <v>0.0000000000110053289448158</v>
+        <v>0.00000000000000696959822809246</v>
       </c>
       <c r="I173" t="n">
-        <v>0.999999999977989</v>
+        <v>0.999999999999986</v>
       </c>
       <c r="J173" t="n">
         <v>9993</v>
@@ -23686,7 +23677,7 @@
         <v>56</v>
       </c>
       <c r="H174" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000346980204133195</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000908122451722972</v>
       </c>
       <c r="I174" t="n">
         <v>1</v>
@@ -23727,13 +23718,13 @@
         <v>56</v>
       </c>
       <c r="H175" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000166709287246273</v>
+        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000047727417431078</v>
       </c>
       <c r="I175" t="n">
         <v>1</v>
       </c>
       <c r="J175" t="n">
-        <v>9991</v>
+        <v>9992</v>
       </c>
       <c r="K175" t="s">
         <v>47</v>
@@ -23768,13 +23759,13 @@
         <v>63</v>
       </c>
       <c r="H176" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000141570289094591</v>
+        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000119572208728018</v>
       </c>
       <c r="I176" t="n">
         <v>1</v>
       </c>
       <c r="J176" t="n">
-        <v>9984</v>
+        <v>9982</v>
       </c>
       <c r="K176" t="s">
         <v>47</v>
@@ -23809,7 +23800,7 @@
         <v>56</v>
       </c>
       <c r="H177" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000352451280950221</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000168426283717792</v>
       </c>
       <c r="I177" t="n">
         <v>1</v>
@@ -23850,7 +23841,7 @@
         <v>63</v>
       </c>
       <c r="H178" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000618886750342356</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000303038505581939</v>
       </c>
       <c r="I178" t="n">
         <v>1</v>
@@ -23891,7 +23882,7 @@
         <v>56</v>
       </c>
       <c r="H179" t="n">
-        <v>0.000000000000000000000000000000000000000000303520830868337</v>
+        <v>0.000000000000000000000000000000000000000986861780966527</v>
       </c>
       <c r="I179" t="n">
         <v>1</v>
@@ -23932,7 +23923,7 @@
         <v>56</v>
       </c>
       <c r="H180" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000571248544341944</v>
+        <v>0.000000000000000000000000000000000000000000000000000000000000000321884547392584</v>
       </c>
       <c r="I180" t="n">
         <v>1</v>
@@ -23973,13 +23964,13 @@
         <v>56</v>
       </c>
       <c r="H181" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000349661888144228</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000744088010370095</v>
       </c>
       <c r="I181" t="n">
         <v>1</v>
       </c>
       <c r="J181" t="n">
-        <v>9976</v>
+        <v>9978</v>
       </c>
       <c r="K181" t="s">
         <v>47</v>
@@ -24014,7 +24005,7 @@
         <v>63</v>
       </c>
       <c r="H182" t="n">
-        <v>0.0000000000000000000000000000000000000000377670449926377</v>
+        <v>0.000000000000000000000000000000000000105629088039657</v>
       </c>
       <c r="I182" t="n">
         <v>1</v>
@@ -24049,16 +24040,16 @@
         <v>56</v>
       </c>
       <c r="F183" t="n">
-        <v>0.999999999980881</v>
+        <v>0.999996129644487</v>
       </c>
       <c r="G183" t="s">
         <v>63</v>
       </c>
       <c r="H183" t="n">
-        <v>0.0000000000191189632844739</v>
+        <v>0.00000387035551336671</v>
       </c>
       <c r="I183" t="n">
-        <v>0.999999999961762</v>
+        <v>0.999992259288973</v>
       </c>
       <c r="J183" t="n">
         <v>10984</v>
@@ -24090,22 +24081,22 @@
         <v>63</v>
       </c>
       <c r="F184" t="n">
-        <v>0.984124827168232</v>
+        <v>0.931552139662621</v>
       </c>
       <c r="G184" t="s">
         <v>56</v>
       </c>
       <c r="H184" t="n">
-        <v>0.0158751728317681</v>
+        <v>0.0684478603373792</v>
       </c>
       <c r="I184" t="n">
-        <v>0.968249654336464</v>
+        <v>0.863104279325242</v>
       </c>
       <c r="J184" t="n">
-        <v>10993</v>
+        <v>10992</v>
       </c>
       <c r="K184" t="s">
-        <v>47</v>
+        <v>150</v>
       </c>
       <c r="L184" t="s">
         <v>48</v>
@@ -24131,16 +24122,16 @@
         <v>63</v>
       </c>
       <c r="F185" t="n">
-        <v>0.999999962646162</v>
+        <v>0.999999872479476</v>
       </c>
       <c r="G185" t="s">
         <v>56</v>
       </c>
       <c r="H185" t="n">
-        <v>0.0000000373538381807721</v>
+        <v>0.000000127520524295597</v>
       </c>
       <c r="I185" t="n">
-        <v>0.999999925292324</v>
+        <v>0.999999744958951</v>
       </c>
       <c r="J185" t="n">
         <v>10992</v>
@@ -24178,7 +24169,7 @@
         <v>56</v>
       </c>
       <c r="H186" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000137222961495538</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000496217428281635</v>
       </c>
       <c r="I186" t="n">
         <v>1</v>
@@ -24219,7 +24210,7 @@
         <v>56</v>
       </c>
       <c r="H187" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000289847596012518</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000547948509607146</v>
       </c>
       <c r="I187" t="n">
         <v>1</v>
@@ -24260,13 +24251,13 @@
         <v>63</v>
       </c>
       <c r="H188" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000044613813380685</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000575235476510115</v>
       </c>
       <c r="I188" t="n">
         <v>1</v>
       </c>
       <c r="J188" t="n">
-        <v>10984</v>
+        <v>10983</v>
       </c>
       <c r="K188" t="s">
         <v>47</v>
@@ -24301,7 +24292,7 @@
         <v>56</v>
       </c>
       <c r="H189" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000583404607311432</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000013065465391547</v>
       </c>
       <c r="I189" t="n">
         <v>1</v>
@@ -24342,7 +24333,7 @@
         <v>63</v>
       </c>
       <c r="H190" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000273936600986573</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000206000626096759</v>
       </c>
       <c r="I190" t="n">
         <v>1</v>
@@ -24383,7 +24374,7 @@
         <v>56</v>
       </c>
       <c r="H191" t="n">
-        <v>0.000000000000000000000000000000000000000000000353924809972507</v>
+        <v>0.00000000000000000000000000000000000000000687080845568202</v>
       </c>
       <c r="I191" t="n">
         <v>1</v>
@@ -24424,13 +24415,13 @@
         <v>56</v>
       </c>
       <c r="H192" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000000000000000917787871688337</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000230938992619241</v>
       </c>
       <c r="I192" t="n">
         <v>1</v>
       </c>
       <c r="J192" t="n">
-        <v>10982</v>
+        <v>10981</v>
       </c>
       <c r="K192" t="s">
         <v>47</v>
@@ -24465,13 +24456,13 @@
         <v>56</v>
       </c>
       <c r="H193" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000430375970744492</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000027671439166465</v>
       </c>
       <c r="I193" t="n">
         <v>1</v>
       </c>
       <c r="J193" t="n">
-        <v>10974</v>
+        <v>10975</v>
       </c>
       <c r="K193" t="s">
         <v>47</v>
@@ -24591,7 +24582,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0000000000000000000000000000000000000000377670449926377</v>
+        <v>0.000000000000000000000000000000000000105629088039657</v>
       </c>
       <c r="N2" t="n">
         <v>1</v>
@@ -24620,13 +24611,13 @@
         <v>56</v>
       </c>
       <c r="D3" t="n">
-        <v>5000</v>
+        <v>11001</v>
       </c>
       <c r="E3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F3" t="n">
         <v>0.666666666666667</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1</v>
       </c>
       <c r="G3" t="n">
         <v>0.5</v>
@@ -24644,13 +24635,13 @@
         <v>11001</v>
       </c>
       <c r="L3" t="n">
-        <v>0.999999999980881</v>
+        <v>0.999996129644487</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0000000000191189632844739</v>
+        <v>0.00000387035551336671</v>
       </c>
       <c r="N3" t="n">
-        <v>0.999999999961762</v>
+        <v>0.999992259288973</v>
       </c>
       <c r="O3" t="s">
         <v>47</v>
@@ -24700,22 +24691,22 @@
         <v>11001</v>
       </c>
       <c r="L4" t="n">
-        <v>0.984124827168232</v>
+        <v>0.931552139662621</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0158751728317681</v>
+        <v>0.0684478603373792</v>
       </c>
       <c r="N4" t="n">
-        <v>0.968249654336464</v>
+        <v>0.863104279325242</v>
       </c>
       <c r="O4" t="s">
-        <v>47</v>
+        <v>150</v>
       </c>
       <c r="P4" t="s">
         <v>48</v>
       </c>
       <c r="Q4" t="n">
-        <v>10993</v>
+        <v>10992</v>
       </c>
       <c r="R4" t="s">
         <v>48</v>
@@ -24732,10 +24723,10 @@
         <v>63</v>
       </c>
       <c r="D5" t="n">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="E5" t="n">
-        <v>0.5</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -24756,13 +24747,13 @@
         <v>11001</v>
       </c>
       <c r="L5" t="n">
-        <v>0.999999962646162</v>
+        <v>0.999999872479476</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0000000373538381807721</v>
+        <v>0.000000127520524295597</v>
       </c>
       <c r="N5" t="n">
-        <v>0.999999925292324</v>
+        <v>0.999999744958951</v>
       </c>
       <c r="O5" t="s">
         <v>47</v>
@@ -24815,7 +24806,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000137222961495538</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000496217428281635</v>
       </c>
       <c r="N6" t="n">
         <v>1</v>
@@ -24871,7 +24862,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000289847596012518</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000547948509607146</v>
       </c>
       <c r="N7" t="n">
         <v>1</v>
@@ -24927,7 +24918,7 @@
         <v>1</v>
       </c>
       <c r="M8" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000044613813380685</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000575235476510115</v>
       </c>
       <c r="N8" t="n">
         <v>1</v>
@@ -24939,7 +24930,7 @@
         <v>48</v>
       </c>
       <c r="Q8" t="n">
-        <v>10984</v>
+        <v>10983</v>
       </c>
       <c r="R8" t="s">
         <v>48</v>
@@ -24983,7 +24974,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000583404607311432</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000013065465391547</v>
       </c>
       <c r="N9" t="n">
         <v>1</v>
@@ -25039,7 +25030,7 @@
         <v>1</v>
       </c>
       <c r="M10" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000273936600986573</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000206000626096759</v>
       </c>
       <c r="N10" t="n">
         <v>1</v>
@@ -25095,7 +25086,7 @@
         <v>1</v>
       </c>
       <c r="M11" t="n">
-        <v>0.000000000000000000000000000000000000000000000353924809972507</v>
+        <v>0.00000000000000000000000000000000000000000687080845568202</v>
       </c>
       <c r="N11" t="n">
         <v>1</v>
@@ -25151,7 +25142,7 @@
         <v>1</v>
       </c>
       <c r="M12" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000000000000000917787871688337</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000230938992619241</v>
       </c>
       <c r="N12" t="n">
         <v>1</v>
@@ -25163,7 +25154,7 @@
         <v>48</v>
       </c>
       <c r="Q12" t="n">
-        <v>10982</v>
+        <v>10981</v>
       </c>
       <c r="R12" t="s">
         <v>48</v>
@@ -25207,7 +25198,7 @@
         <v>1</v>
       </c>
       <c r="M13" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000430375970744492</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000027671439166465</v>
       </c>
       <c r="N13" t="n">
         <v>1</v>
@@ -25219,7 +25210,7 @@
         <v>48</v>
       </c>
       <c r="Q13" t="n">
-        <v>10974</v>
+        <v>10975</v>
       </c>
       <c r="R13" t="s">
         <v>48</v>
@@ -27470,10 +27461,10 @@
         <v>1</v>
       </c>
       <c r="G72" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H72" t="n">
-        <v>0.00000000000000000000000000000024342522668168</v>
+        <v>0.0000000000000000000000000000000462446810801965</v>
       </c>
       <c r="I72" t="n">
         <v>1</v>
@@ -27505,25 +27496,25 @@
         <v>51</v>
       </c>
       <c r="E73" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="F73" t="n">
-        <v>0.870225012679012</v>
+        <v>0.783632514541674</v>
       </c>
       <c r="G73" t="s">
         <v>52</v>
       </c>
       <c r="H73" t="n">
-        <v>0.129774987320978</v>
+        <v>0.216367485458323</v>
       </c>
       <c r="I73" t="n">
-        <v>0.740450025358034</v>
+        <v>0.567265029083351</v>
       </c>
       <c r="J73" t="n">
         <v>500</v>
       </c>
       <c r="K73" t="s">
-        <v>153</v>
+        <v>90</v>
       </c>
       <c r="L73" t="s">
         <v>48</v>
@@ -27552,10 +27543,10 @@
         <v>1</v>
       </c>
       <c r="G74" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H74" t="n">
-        <v>0.00000000000000000000000000000000000000300728468201661</v>
+        <v>0.000000000000000000000000000000000000000872373303422011</v>
       </c>
       <c r="I74" t="n">
         <v>1</v>
@@ -27590,16 +27581,16 @@
         <v>49</v>
       </c>
       <c r="F75" t="n">
-        <v>0.999999999999978</v>
+        <v>0.999999999999973</v>
       </c>
       <c r="G75" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H75" t="n">
-        <v>0.0000000000000216397667274875</v>
+        <v>0.0000000000000271671241370854</v>
       </c>
       <c r="I75" t="n">
-        <v>0.999999999999957</v>
+        <v>0.999999999999946</v>
       </c>
       <c r="J75" t="n">
         <v>499</v>
@@ -27631,16 +27622,16 @@
         <v>49</v>
       </c>
       <c r="F76" t="n">
-        <v>0.999995572344271</v>
+        <v>0.999999287333286</v>
       </c>
       <c r="G76" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H76" t="n">
-        <v>0.0000044276557291108</v>
+        <v>0.000000712666713728956</v>
       </c>
       <c r="I76" t="n">
-        <v>0.999991144688542</v>
+        <v>0.999998574666572</v>
       </c>
       <c r="J76" t="n">
         <v>500</v>
@@ -27672,16 +27663,16 @@
         <v>49</v>
       </c>
       <c r="F77" t="n">
-        <v>0.999998324811452</v>
+        <v>0.999999780354469</v>
       </c>
       <c r="G77" t="s">
         <v>52</v>
       </c>
       <c r="H77" t="n">
-        <v>0.00000126637763426342</v>
+        <v>0.000000141981609489582</v>
       </c>
       <c r="I77" t="n">
-        <v>0.999997058433818</v>
+        <v>0.999999638372859</v>
       </c>
       <c r="J77" t="n">
         <v>500</v>
@@ -27716,10 +27707,10 @@
         <v>1</v>
       </c>
       <c r="G78" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H78" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000831697423330759</v>
+        <v>0.000000000000000000000000000000000000000000000000000182587688543977</v>
       </c>
       <c r="I78" t="n">
         <v>1</v>
@@ -27757,10 +27748,10 @@
         <v>1</v>
       </c>
       <c r="G79" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H79" t="n">
-        <v>0.00000000000000000000000000000000000000000000000193925997760556</v>
+        <v>0.00000000000000000000000000000000000000000000000732745298134101</v>
       </c>
       <c r="I79" t="n">
         <v>1</v>
@@ -27798,10 +27789,10 @@
         <v>1</v>
       </c>
       <c r="G80" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H80" t="n">
-        <v>0.00000000000000000196167827701144</v>
+        <v>0.00000000000000000119052760836764</v>
       </c>
       <c r="I80" t="n">
         <v>1</v>
@@ -27839,10 +27830,10 @@
         <v>1</v>
       </c>
       <c r="G81" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H81" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000038725495925259</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000175179425015209</v>
       </c>
       <c r="I81" t="n">
         <v>1</v>
@@ -27880,10 +27871,10 @@
         <v>1</v>
       </c>
       <c r="G82" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H82" t="n">
-        <v>0.00000000000000000000000109920404502996</v>
+        <v>0.0000000000000000000000000446078114038661</v>
       </c>
       <c r="I82" t="n">
         <v>1</v>
@@ -27918,16 +27909,16 @@
         <v>49</v>
       </c>
       <c r="F83" t="n">
-        <v>0.999999999988209</v>
+        <v>0.999999999999813</v>
       </c>
       <c r="G83" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H83" t="n">
-        <v>0.0000000000117911584893823</v>
+        <v>0.00000000000018748859362629</v>
       </c>
       <c r="I83" t="n">
-        <v>0.999999999976418</v>
+        <v>0.999999999999625</v>
       </c>
       <c r="J83" t="n">
         <v>999</v>
@@ -27959,16 +27950,16 @@
         <v>49</v>
       </c>
       <c r="F84" t="n">
-        <v>0.999999999983811</v>
+        <v>0.999999999906909</v>
       </c>
       <c r="G84" t="s">
         <v>52</v>
       </c>
       <c r="H84" t="n">
-        <v>0.0000000000161893856573261</v>
+        <v>0.0000000000930912053265774</v>
       </c>
       <c r="I84" t="n">
-        <v>0.999999999967621</v>
+        <v>0.999999999813817</v>
       </c>
       <c r="J84" t="n">
         <v>999</v>
@@ -28006,7 +27997,7 @@
         <v>52</v>
       </c>
       <c r="H85" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000503794353398441</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000671710253182587</v>
       </c>
       <c r="I85" t="n">
         <v>1</v>
@@ -28047,7 +28038,7 @@
         <v>52</v>
       </c>
       <c r="H86" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000331998927808627</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000010968472181666</v>
       </c>
       <c r="I86" t="n">
         <v>1</v>
@@ -28088,7 +28079,7 @@
         <v>49</v>
       </c>
       <c r="H87" t="n">
-        <v>0.000000000000000000000000000000000433171192083059</v>
+        <v>0.000000000000000000000000000000000000143755501845078</v>
       </c>
       <c r="I87" t="n">
         <v>1</v>
@@ -28126,10 +28117,10 @@
         <v>1</v>
       </c>
       <c r="G88" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H88" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000273620022825877</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000128390663951282</v>
       </c>
       <c r="I88" t="n">
         <v>1</v>
@@ -28170,7 +28161,7 @@
         <v>52</v>
       </c>
       <c r="H89" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000679449883353685</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000349929645280327</v>
       </c>
       <c r="I89" t="n">
         <v>1</v>
@@ -28208,10 +28199,10 @@
         <v>1</v>
       </c>
       <c r="G90" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H90" t="n">
-        <v>0.0000000000000000000000000000233596002006557</v>
+        <v>0.0000000000000000000000000116782818278807</v>
       </c>
       <c r="I90" t="n">
         <v>1</v>
@@ -28252,7 +28243,7 @@
         <v>52</v>
       </c>
       <c r="H91" t="n">
-        <v>0.00000000000000000000000185006725856613</v>
+        <v>0.00000000000000000000000165268166350742</v>
       </c>
       <c r="I91" t="n">
         <v>1</v>
@@ -28293,7 +28284,7 @@
         <v>52</v>
       </c>
       <c r="H92" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000190639737199453</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000909473821225966</v>
       </c>
       <c r="I92" t="n">
         <v>1</v>
@@ -28334,13 +28325,13 @@
         <v>52</v>
       </c>
       <c r="H93" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000641996477757158</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000483095182196647</v>
       </c>
       <c r="I93" t="n">
         <v>1</v>
       </c>
       <c r="J93" t="n">
-        <v>4993</v>
+        <v>4992</v>
       </c>
       <c r="K93" t="s">
         <v>47</v>
@@ -28375,7 +28366,7 @@
         <v>49</v>
       </c>
       <c r="H94" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000260849399112077</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000115863210339421</v>
       </c>
       <c r="I94" t="n">
         <v>1</v>
@@ -28416,7 +28407,7 @@
         <v>52</v>
       </c>
       <c r="H95" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000892425189499396</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000021373615600613</v>
       </c>
       <c r="I95" t="n">
         <v>1</v>
@@ -28457,13 +28448,13 @@
         <v>52</v>
       </c>
       <c r="H96" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000522914589620841</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000127053657805336</v>
       </c>
       <c r="I96" t="n">
         <v>1</v>
       </c>
       <c r="J96" t="n">
-        <v>4988</v>
+        <v>4987</v>
       </c>
       <c r="K96" t="s">
         <v>47</v>
@@ -28495,10 +28486,10 @@
         <v>1</v>
       </c>
       <c r="G97" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H97" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000022479083343352</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000145435676914854</v>
       </c>
       <c r="I97" t="n">
         <v>1</v>
@@ -28539,7 +28530,7 @@
         <v>52</v>
       </c>
       <c r="H98" t="n">
-        <v>0.000000000000000000000000000000000000499311495165198</v>
+        <v>0.00000000000000000000000000000000000000133219821150407</v>
       </c>
       <c r="I98" t="n">
         <v>1</v>
@@ -28580,13 +28571,13 @@
         <v>52</v>
       </c>
       <c r="H99" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000268513136827898</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000050023654136164</v>
       </c>
       <c r="I99" t="n">
         <v>1</v>
       </c>
       <c r="J99" t="n">
-        <v>4993</v>
+        <v>4992</v>
       </c>
       <c r="K99" t="s">
         <v>47</v>
@@ -28621,13 +28612,13 @@
         <v>52</v>
       </c>
       <c r="H100" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000327571519567526</v>
+        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000311081808925194</v>
       </c>
       <c r="I100" t="n">
         <v>1</v>
       </c>
       <c r="J100" t="n">
-        <v>9983</v>
+        <v>9984</v>
       </c>
       <c r="K100" t="s">
         <v>47</v>
@@ -28662,13 +28653,13 @@
         <v>49</v>
       </c>
       <c r="H101" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000467698538831469</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000498489578873013</v>
       </c>
       <c r="I101" t="n">
         <v>1</v>
       </c>
       <c r="J101" t="n">
-        <v>9985</v>
+        <v>9984</v>
       </c>
       <c r="K101" t="s">
         <v>47</v>
@@ -28703,7 +28694,7 @@
         <v>52</v>
       </c>
       <c r="H102" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000171716605634234</v>
+        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000069583498563995</v>
       </c>
       <c r="I102" t="n">
         <v>1</v>
@@ -28744,13 +28735,13 @@
         <v>52</v>
       </c>
       <c r="H103" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000295201842551035</v>
+        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000271937669517401</v>
       </c>
       <c r="I103" t="n">
         <v>1</v>
       </c>
       <c r="J103" t="n">
-        <v>9976</v>
+        <v>9975</v>
       </c>
       <c r="K103" t="s">
         <v>47</v>
@@ -28785,13 +28776,13 @@
         <v>52</v>
       </c>
       <c r="H104" t="n">
-        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000164498961264595</v>
+        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000266880867782718</v>
       </c>
       <c r="I104" t="n">
         <v>1</v>
       </c>
       <c r="J104" t="n">
-        <v>9987</v>
+        <v>9988</v>
       </c>
       <c r="K104" t="s">
         <v>47</v>
@@ -28826,13 +28817,13 @@
         <v>52</v>
       </c>
       <c r="H105" t="n">
-        <v>0.000000000000000000000000000000000000000000000131252082568585</v>
+        <v>0.0000000000000000000000000000000000000000000235622115545669</v>
       </c>
       <c r="I105" t="n">
         <v>1</v>
       </c>
       <c r="J105" t="n">
-        <v>9990</v>
+        <v>9991</v>
       </c>
       <c r="K105" t="s">
         <v>47</v>
@@ -28867,13 +28858,13 @@
         <v>52</v>
       </c>
       <c r="H106" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000272524576644728</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000982154472742514</v>
       </c>
       <c r="I106" t="n">
         <v>1</v>
       </c>
       <c r="J106" t="n">
-        <v>9988</v>
+        <v>9987</v>
       </c>
       <c r="K106" t="s">
         <v>47</v>
@@ -28908,13 +28899,13 @@
         <v>52</v>
       </c>
       <c r="H107" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000500495349557371</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000165888946553371</v>
       </c>
       <c r="I107" t="n">
         <v>1</v>
       </c>
       <c r="J107" t="n">
-        <v>11069</v>
+        <v>11070</v>
       </c>
       <c r="K107" t="s">
         <v>47</v>
@@ -28949,13 +28940,13 @@
         <v>49</v>
       </c>
       <c r="H108" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000176351078870957</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000445363581161422</v>
       </c>
       <c r="I108" t="n">
         <v>1</v>
       </c>
       <c r="J108" t="n">
-        <v>11071</v>
+        <v>11070</v>
       </c>
       <c r="K108" t="s">
         <v>47</v>
@@ -28990,13 +28981,13 @@
         <v>52</v>
       </c>
       <c r="H109" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000129176415778798</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000270836020877928</v>
       </c>
       <c r="I109" t="n">
         <v>1</v>
       </c>
       <c r="J109" t="n">
-        <v>11074</v>
+        <v>11075</v>
       </c>
       <c r="K109" t="s">
         <v>47</v>
@@ -29031,13 +29022,13 @@
         <v>52</v>
       </c>
       <c r="H110" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000489105172250268</v>
+        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000156505623275388</v>
       </c>
       <c r="I110" t="n">
         <v>1</v>
       </c>
       <c r="J110" t="n">
-        <v>11060</v>
+        <v>11059</v>
       </c>
       <c r="K110" t="s">
         <v>47</v>
@@ -29072,13 +29063,13 @@
         <v>52</v>
       </c>
       <c r="H111" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000182743004401083</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000829502186312922</v>
       </c>
       <c r="I111" t="n">
         <v>1</v>
       </c>
       <c r="J111" t="n">
-        <v>11073</v>
+        <v>11074</v>
       </c>
       <c r="K111" t="s">
         <v>47</v>
@@ -29113,13 +29104,13 @@
         <v>52</v>
       </c>
       <c r="H112" t="n">
-        <v>0.00000000000000000000000000000000000000000000000416303022146296</v>
+        <v>0.00000000000000000000000000000000000000000000142759576129688</v>
       </c>
       <c r="I112" t="n">
         <v>1</v>
       </c>
       <c r="J112" t="n">
-        <v>11076</v>
+        <v>11077</v>
       </c>
       <c r="K112" t="s">
         <v>47</v>
@@ -29154,13 +29145,13 @@
         <v>52</v>
       </c>
       <c r="H113" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000037308430829846</v>
+        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000377934333794494</v>
       </c>
       <c r="I113" t="n">
         <v>1</v>
       </c>
       <c r="J113" t="n">
-        <v>11073</v>
+        <v>11072</v>
       </c>
       <c r="K113" t="s">
         <v>47</v>
@@ -29280,7 +29271,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000500495349557371</v>
+        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000165888946553371</v>
       </c>
       <c r="N2" t="n">
         <v>1</v>
@@ -29292,7 +29283,7 @@
         <v>48</v>
       </c>
       <c r="Q2" t="n">
-        <v>11069</v>
+        <v>11070</v>
       </c>
       <c r="R2" t="s">
         <v>48</v>
@@ -29336,7 +29327,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000176351078870957</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000445363581161422</v>
       </c>
       <c r="N3" t="n">
         <v>1</v>
@@ -29348,7 +29339,7 @@
         <v>48</v>
       </c>
       <c r="Q3" t="n">
-        <v>11071</v>
+        <v>11070</v>
       </c>
       <c r="R3" t="s">
         <v>48</v>
@@ -29392,7 +29383,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000129176415778798</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000270836020877928</v>
       </c>
       <c r="N4" t="n">
         <v>1</v>
@@ -29404,7 +29395,7 @@
         <v>48</v>
       </c>
       <c r="Q4" t="n">
-        <v>11074</v>
+        <v>11075</v>
       </c>
       <c r="R4" t="s">
         <v>48</v>
@@ -29448,7 +29439,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000489105172250268</v>
+        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000156505623275388</v>
       </c>
       <c r="N5" t="n">
         <v>1</v>
@@ -29460,7 +29451,7 @@
         <v>48</v>
       </c>
       <c r="Q5" t="n">
-        <v>11060</v>
+        <v>11059</v>
       </c>
       <c r="R5" t="s">
         <v>48</v>
@@ -29504,7 +29495,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000182743004401083</v>
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000829502186312922</v>
       </c>
       <c r="N6" t="n">
         <v>1</v>
@@ -29516,7 +29507,7 @@
         <v>48</v>
       </c>
       <c r="Q6" t="n">
-        <v>11073</v>
+        <v>11074</v>
       </c>
       <c r="R6" t="s">
         <v>48</v>
@@ -29560,7 +29551,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>0.00000000000000000000000000000000000000000000000416303022146296</v>
+        <v>0.00000000000000000000000000000000000000000000142759576129688</v>
       </c>
       <c r="N7" t="n">
         <v>1</v>
@@ -29572,7 +29563,7 @@
         <v>48</v>
       </c>
       <c r="Q7" t="n">
-        <v>11076</v>
+        <v>11077</v>
       </c>
       <c r="R7" t="s">
         <v>48</v>
@@ -29616,7 +29607,7 @@
         <v>1</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000037308430829846</v>
+        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000377934333794494</v>
       </c>
       <c r="N8" t="n">
         <v>1</v>
@@ -29628,7 +29619,7 @@
         <v>48</v>
       </c>
       <c r="Q8" t="n">
-        <v>11073</v>
+        <v>11072</v>
       </c>
       <c r="R8" t="s">
         <v>48</v>
@@ -29650,170 +29641,170 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B1" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B2" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B3" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B4" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B5" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B7" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="B10" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B11" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B12" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B13" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B14" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="B15" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="B16" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B17" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B18" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B19" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B20" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="B21" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="22">
@@ -29821,55 +29812,55 @@
         <v>126</v>
       </c>
       <c r="B22" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B23" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B24" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="B25" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B26" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B27" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B28" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>

</xml_diff>